<commit_message>
fix(seed): GNDEC student names vary across sections; teachers are Dr. / Prof. (clean login emails)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo-data/GNDEC/GNDEC_1_AS.xlsx
+++ b/docs/demo-data/GNDEC/GNDEC_1_AS.xlsx
@@ -789,7 +789,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Er. Navneet Ahluwalia</t>
+          <t>Dr. Navneet Ahluwalia</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -804,7 +804,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dr. Amandeep Kohli</t>
+          <t>Prof. Amandeep Kohli</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -819,7 +819,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Prof. Rupinder Jindal</t>
+          <t>Dr. Rupinder Jindal</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -834,7 +834,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Er. Simranjit Randhawa</t>
+          <t>Prof. Simranjit Randhawa</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -879,7 +879,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Er. Ravneet Mittal</t>
+          <t>Dr. Ravneet Mittal</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -894,7 +894,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dr. Jagmeet Cheema</t>
+          <t>Prof. Jagmeet Cheema</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -909,7 +909,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Prof. Tejinder Mann</t>
+          <t>Dr. Tejinder Mann</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -924,7 +924,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Er. Manveer Khanna</t>
+          <t>Prof. Manveer Khanna</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -969,7 +969,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Er. Prabhjot Toor</t>
+          <t>Dr. Prabhjot Toor</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -984,7 +984,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dr. Ishpreet Bedi</t>
+          <t>Prof. Ishpreet Bedi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -999,7 +999,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Prof. Gagandeep Anand</t>
+          <t>Dr. Gagandeep Anand</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1014,7 +1014,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Er. Rajvir Garg</t>
+          <t>Prof. Rajvir Garg</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Er. Nitin Bhalla</t>
+          <t>Dr. Nitin Bhalla</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1074,7 +1074,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dr. Pooja Bansal</t>
+          <t>Prof. Pooja Bansal</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1089,7 +1089,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Prof. Sanjeev Dhaliwal</t>
+          <t>Dr. Sanjeev Dhaliwal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1104,7 +1104,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Er. Meenu Gill</t>
+          <t>Prof. Meenu Gill</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1149,7 +1149,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Er. Aman Bains</t>
+          <t>Dr. Aman Bains</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1164,7 +1164,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dr. Nidhi Brar</t>
+          <t>Prof. Nidhi Brar</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1500,7 +1500,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Er. Navneet Ahluwalia</t>
+          <t>Dr. Navneet Ahluwalia</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1515,7 +1515,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dr. Amandeep Kohli</t>
+          <t>Prof. Amandeep Kohli</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1530,7 +1530,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Prof. Rupinder Jindal</t>
+          <t>Dr. Rupinder Jindal</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1545,7 +1545,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Er. Simranjit Randhawa</t>
+          <t>Prof. Simranjit Randhawa</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1590,7 +1590,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Er. Ravneet Mittal</t>
+          <t>Dr. Ravneet Mittal</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1605,7 +1605,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dr. Jagmeet Cheema</t>
+          <t>Prof. Jagmeet Cheema</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1620,7 +1620,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Prof. Tejinder Mann</t>
+          <t>Dr. Tejinder Mann</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1635,7 +1635,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Er. Manveer Khanna</t>
+          <t>Prof. Manveer Khanna</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1680,7 +1680,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Er. Prabhjot Toor</t>
+          <t>Dr. Prabhjot Toor</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1695,7 +1695,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Dr. Ishpreet Bedi</t>
+          <t>Prof. Ishpreet Bedi</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1710,7 +1710,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Prof. Gagandeep Anand</t>
+          <t>Dr. Gagandeep Anand</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1725,7 +1725,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Er. Rajvir Garg</t>
+          <t>Prof. Rajvir Garg</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1770,7 +1770,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Er. Nitin Bhalla</t>
+          <t>Dr. Nitin Bhalla</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1785,7 +1785,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dr. Pooja Bansal</t>
+          <t>Prof. Pooja Bansal</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1800,7 +1800,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Prof. Sanjeev Dhaliwal</t>
+          <t>Dr. Sanjeev Dhaliwal</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1815,7 +1815,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Er. Meenu Gill</t>
+          <t>Prof. Meenu Gill</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1860,7 +1860,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Er. Aman Bains</t>
+          <t>Dr. Aman Bains</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1875,7 +1875,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Dr. Nidhi Brar</t>
+          <t>Prof. Nidhi Brar</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1890,7 +1890,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Dr. Amandeep Kohli</t>
+          <t>Prof. Amandeep Kohli</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">

</xml_diff>

<commit_message>
fix(seed): GNDEC first-year halls belong to Applied Sciences so the uploads are complete
Lecture theatres, drawing halls and workshops were shared rooms, which no department
file carries, so a college built from the files lacked them. They now belong to
Applied Sciences (uploaded first). Tested the user's path on a local copy: new
college, GNDEC time grid + 5 departments in Setup, upload the 5 files in order
(0 row errors each), pre-check clean, generate 557 classes with 0 clashes, publish.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/demo-data/GNDEC/GNDEC_1_AS.xlsx
+++ b/docs/demo-data/GNDEC/GNDEC_1_AS.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -472,178 +472,185 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>then CSE, IT, ME and CE. Shared halls, the JPAL hour and the final-year CSE elective are set up by</t>
+          <t>then CSE, IT, ME and CE. Its file also has the lecture theatres, drawing halls and workshops of</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>the College Admin (they are already in the built-in GNDEC demo college).</t>
+          <t>first year. Not in the files: the JPAL hour and the final-year CSE elective (they need a student list</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>per group; they are in the built-in GNDEC demo college).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Timetabl.ai: one department's data</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-    </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Fill one file per department and upload it on the department's page (Setup &gt; Departments &gt; Upload Excel).</t>
-        </is>
-      </c>
+      <c r="A9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Fill one file per department and upload it on the department's page (Setup &gt; Departments &gt; Upload Excel).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Rows are checked before anything is saved; problems are shown row by row. A '*' marks a required column.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Sections: one row per section (a group of students who always sit together).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Section: its name, e.g. D2CS-A. Year: 1-4. Students: how many. Shift: the shift name from Setup (e.g. Day).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Section: its name, e.g. D2CS-A. Year: 1-4. Students: how many. Shift: the shift name from Setup (e.g. Day).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Lab batches: how the section splits for labs, e.g. 'A1:30, A2:30' (name:students). Empty = whole section.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Teachers: one row per teacher of the department.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t xml:space="preserve">  Name, Email (their login), Shifts (one or more shift names, comma separated), Max periods per day (default 5).</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Subjects: one row per subject the department teaches.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Code, Name, Year, Lectures per week, Labs per week (lab blocks; one block = the college's lab length, e.g. 2 periods),</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Code, Name, Year, Lectures per week, Labs per week (lab blocks; one block = the college's lab length, e.g. 2 periods),</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Lab equipment: what the lab room must have, e.g. computers. It must match a lab room's Equipment.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Can teach: which subjects each teacher can teach. Preference 1 = first choice, 2 = could also teach it.</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t xml:space="preserve">  Used for teacher suggestions and to find a substitute when a teacher is on leave.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Classes: one row per class. Subject code, Sections (several separated by commas = one combined class),</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Type (Lecture or Lab), Batch ('all' = one lab for each lab batch, or one batch name), Teacher (may be empty).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A teacher or subject of another department (e.g. Applied Sciences for first-year maths) can be named too,</t>
+          <t xml:space="preserve">  Type (Lecture or Lab), Batch ('all' = one lab for each lab batch, or one batch name), Teacher (may be empty).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t xml:space="preserve">  A teacher or subject of another department (e.g. Applied Sciences for first-year maths) can be named too,</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t xml:space="preserve">  once that department's file is uploaded: upload Applied Sciences first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Students: Roll no, Name, Email (their login; first password = roll number), Section, Batch.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
+          <t>Students: Roll no, Name, Email (their login; first password = roll number), Section, Batch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
           <t>Rooms: rooms this department owns. Type: Lecture, Lab or Seminar. Seats. Equipment for labs.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Shared halls (lecture theatres, seminar hall, drawing halls, workshops) are added by the College Admin in Setup.</t>
-        </is>
-      </c>
-    </row>
     <row r="29">
-      <c r="A29" t="inlineStr"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Rooms every department may use (e.g. a seminar hall) are added by the College Admin in Setup as shared rooms.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Not in this file: the time grid, lunch window, holidays, electives and pooled groups (e.g. JPAL),</t>
-        </is>
-      </c>
+      <c r="A30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
+        <is>
+          <t>Not in this file: the time grid, lunch window, holidays, electives and pooled groups (e.g. JPAL),</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
         <is>
           <t>rules and shared rooms. The College Admin sets those in Setup.</t>
         </is>
@@ -2131,7 +2138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2171,7 +2178,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A-101</t>
+          <t>Lecture Theatre LT-1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -2180,13 +2187,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>70</v>
+        <v>150</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A-102</t>
+          <t>Lecture Theatre LT-2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2195,46 +2202,156 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>70</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Physics Lab</t>
+          <t>A-101</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Lab</t>
+          <t>Lecture</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>32</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>physics</t>
-        </is>
+        <v>70</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>A-102</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Physics Lab</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>32</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>physics</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Basic Electrical Lab</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Lab</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="C7" t="n">
         <v>32</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>electrical</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Drawing Hall-1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>32</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Drawing Hall-2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>32</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>drawing</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Central Workshop-1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>32</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>workshop</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Central Workshop-2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Lab</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>32</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>workshop</t>
         </is>
       </c>
     </row>

</xml_diff>